<commit_message>
Address 3rd review: Q1 SQL source names + remove leftover "4 Jul"
Two workbook-polish items from the latest review (the Q2 CART and Q5
enrollment-span findings were already resolved on this branch in the prior
commit, which post-dated the reviewed main).

- Q1 real-patient extraction SQL: switch bare <cdm>.t_rx / <cdm>.t_medical to
  the cdm_src()-resolved quarterly names (t_rx_2025q2 / t_medical_2025q2) with
  an explanatory comment, consistent with the Q5 tab — avoids a handoff trap
  for whoever runs it in Databricks.
- Read Me: replace the remaining "Julia, 4 Jul 2026" heading with a
  folder-anchored reference (Questions/July 5 2026), so no stale date remains.

Workbook rebuilt from the committed bundle via build_workbook.py.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Mb2U6kDRP7ZNyny6V62gi
</commit_message>
<xml_diff>
--- a/Questions/July 5 2026/julia_july5_answers.xlsx
+++ b/Questions/July 5 2026/julia_july5_answers.xlsx
@@ -766,7 +766,7 @@
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>The five questions (Julia, 4 Jul 2026)</t>
+          <t>The five questions (Julia, chat forwarded — Questions/July 5 2026)</t>
         </is>
       </c>
     </row>
@@ -1883,15 +1883,17 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="174" customHeight="1">
+    <row r="24" ht="202" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>-- 1. Raw pharmacy + medical claims for one patient (chronological)
-SELECT 'pharmacy' src, FILL_DT dt, NDC code, DAYS_SUP FROM &lt;cdm&gt;.t_rx      WHERE PATID = :pid
+          <t>-- CDM tables resolve through cdm_src() to the quarterly names when USE_QUARTERLY_TABLES=TRUE,
+-- e.g. cdm_src('rx') -&gt; &lt;cdm&gt;.t_rx_2025q2, cdm_src('medical') -&gt; &lt;cdm&gt;.t_medical_2025q2.
+-- 1. Raw pharmacy + medical claims for one patient (chronological)
+SELECT 'pharmacy' src, FILL_DT dt, NDC code, DAYS_SUP FROM &lt;cdm&gt;.t_rx_2025q2      WHERE PATID = :pid  -- cdm_src('rx')
 UNION ALL
-SELECT 'medical'  src, FST_DT  dt, PROC_CD, NULL   FROM &lt;cdm&gt;.t_medical    WHERE PATID = :pid
+SELECT 'medical'  src, FST_DT  dt, PROC_CD, NULL   FROM &lt;cdm&gt;.t_medical_2025q2    WHERE PATID = :pid  -- cdm_src('medical')
 ORDER BY dt;
--- 2. The MAP segments the engine built, and the final line assignment
+-- 2. The MAP segments the engine built, and the final line assignment (work schema)
 SELECT * FROM &lt;work&gt;.MAP_STACKED WHERE PATID = :pid ORDER BY MAP_START_DT;
 SELECT LOT_NUM, LOT_START_DT, LOT_START_TYPE, LOT_BASE_MEDS, LOT_BASE_END_DT,
        LOT_BASE_END_REASON, LOT_ALLO_LOT_FLG, LOT_CART_LOT_FLG,

</xml_diff>